<commit_message>
fix bug api find all asset
</commit_message>
<xml_diff>
--- a/src/main/resources/static/reports/37_C53 - HD_Bien ban kiem ke TSCD.xlsx
+++ b/src/main/resources/static/reports/37_C53 - HD_Bien ban kiem ke TSCD.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\Project_BK\csvc-hust\src\main\resources\static\reports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\Báo cáo-20241024T034450Z-001\Báo cáo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21BCECEE-A838-4B08-B0E3-0E5F721BD162}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{367F8D97-7FEB-4EB7-B195-09C9B2958CBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6BF27037-C3F5-45D1-9348-21FE8AF99BBC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{6BF27037-C3F5-45D1-9348-21FE8AF99BBC}"/>
   </bookViews>
   <sheets>
     <sheet name="Biên bản kiểm kê TSCĐ" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="38">
   <si>
     <t>Đơn vị :................................</t>
   </si>
@@ -117,6 +117,24 @@
   </si>
   <si>
     <t>E</t>
+  </si>
+  <si>
+    <t>Thủ trưởng đơn vị</t>
+  </si>
+  <si>
+    <t>Kế toán trưởng</t>
+  </si>
+  <si>
+    <t>Trưởng Ban kiểm kê</t>
+  </si>
+  <si>
+    <t>(Ý kiến giải quyết số chênh lệch)</t>
+  </si>
+  <si>
+    <t>(Ký, họ tên, đóng dấu)</t>
+  </si>
+  <si>
+    <t>(Ký, họ tên)</t>
   </si>
   <si>
     <t>Số:............</t>
@@ -323,7 +341,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -341,9 +359,39 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -353,45 +401,25 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -730,140 +758,140 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:N25"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.28515625" style="6" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" style="6" customWidth="1"/>
-    <col min="3" max="14" width="10.5703125" style="6" customWidth="1"/>
-    <col min="15" max="16384" width="8.7109375" style="6"/>
+    <col min="1" max="1" width="6.21875" style="6" customWidth="1"/>
+    <col min="2" max="2" width="18.77734375" style="6" customWidth="1"/>
+    <col min="3" max="14" width="10.5546875" style="6" customWidth="1"/>
+    <col min="15" max="16384" width="8.77734375" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="J1" s="17" t="s">
-        <v>28</v>
-      </c>
-      <c r="K1" s="17"/>
-      <c r="L1" s="17"/>
-      <c r="M1" s="17"/>
-      <c r="N1" s="17"/>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J1" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="J2" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="K2" s="18"/>
-      <c r="L2" s="18"/>
-      <c r="M2" s="18"/>
-      <c r="N2" s="18"/>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J2" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="9"/>
+      <c r="N2" s="9"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="19" t="s">
-        <v>30</v>
-      </c>
-      <c r="K3" s="19"/>
-      <c r="L3" s="19"/>
-      <c r="M3" s="19"/>
-      <c r="N3" s="19"/>
-    </row>
-    <row r="5" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="20" t="s">
+      <c r="J3" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="K3" s="10"/>
+      <c r="L3" s="10"/>
+      <c r="M3" s="10"/>
+      <c r="N3" s="10"/>
+    </row>
+    <row r="5" spans="1:14" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A5" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20"/>
-      <c r="H5" s="20"/>
-      <c r="I5" s="20"/>
-      <c r="J5" s="20"/>
-      <c r="K5" s="20"/>
-      <c r="L5" s="20"/>
-      <c r="M5" s="20"/>
-      <c r="N5" s="20"/>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="M6" s="21" t="s">
-        <v>27</v>
-      </c>
-      <c r="N6" s="21"/>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M6" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="N6" s="8"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="22.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="B13" s="22" t="s">
+    <row r="13" spans="1:14" ht="22.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="22" t="s">
+      <c r="C13" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="D13" s="22" t="s">
+      <c r="D13" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E13" s="14" t="s">
+      <c r="E13" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="F13" s="15"/>
-      <c r="G13" s="16"/>
-      <c r="H13" s="14" t="s">
+      <c r="F13" s="14"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="I13" s="15"/>
-      <c r="J13" s="16"/>
-      <c r="K13" s="14" t="s">
+      <c r="I13" s="14"/>
+      <c r="J13" s="15"/>
+      <c r="K13" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="L13" s="15"/>
-      <c r="M13" s="16"/>
-      <c r="N13" s="7"/>
-    </row>
-    <row r="14" spans="1:14" ht="40.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="23"/>
-      <c r="B14" s="23"/>
-      <c r="C14" s="23"/>
-      <c r="D14" s="23"/>
-      <c r="E14" s="8" t="s">
+      <c r="L13" s="14"/>
+      <c r="M13" s="15"/>
+      <c r="N13" s="16"/>
+    </row>
+    <row r="14" spans="1:14" ht="40.200000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="17"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="18" t="s">
         <v>15</v>
       </c>
       <c r="F14" s="5" t="s">
@@ -872,73 +900,73 @@
       <c r="G14" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H14" s="8" t="s">
+      <c r="H14" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="8" t="s">
+      <c r="I14" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="J14" s="8" t="s">
+      <c r="J14" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="K14" s="8" t="s">
+      <c r="K14" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="L14" s="8" t="s">
+      <c r="L14" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="M14" s="8" t="s">
+      <c r="M14" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="N14" s="8" t="s">
+      <c r="N14" s="18" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="9" t="s">
+    <row r="15" spans="1:14" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="E15" s="10">
+      <c r="E15" s="20">
         <v>1</v>
       </c>
-      <c r="F15" s="10">
+      <c r="F15" s="20">
         <v>2</v>
       </c>
-      <c r="G15" s="10">
+      <c r="G15" s="20">
         <v>3</v>
       </c>
-      <c r="H15" s="10">
+      <c r="H15" s="20">
         <v>4</v>
       </c>
-      <c r="I15" s="10">
+      <c r="I15" s="20">
         <v>5</v>
       </c>
-      <c r="J15" s="10">
+      <c r="J15" s="20">
         <v>6</v>
       </c>
-      <c r="K15" s="10">
+      <c r="K15" s="20">
         <v>7</v>
       </c>
-      <c r="L15" s="10">
+      <c r="L15" s="20">
         <v>8</v>
       </c>
-      <c r="M15" s="10">
+      <c r="M15" s="20">
         <v>9</v>
       </c>
-      <c r="N15" s="10" t="s">
+      <c r="N15" s="20" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -954,7 +982,7 @@
       <c r="M16" s="3"/>
       <c r="N16" s="3"/>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" s="2"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -970,7 +998,7 @@
       <c r="M17" s="3"/>
       <c r="N17" s="3"/>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -986,7 +1014,7 @@
       <c r="M18" s="3"/>
       <c r="N18" s="3"/>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -1002,7 +1030,7 @@
       <c r="M19" s="3"/>
       <c r="N19" s="3"/>
     </row>
-    <row r="20" spans="1:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -1018,7 +1046,7 @@
       <c r="M20" s="3"/>
       <c r="N20" s="3"/>
     </row>
-    <row r="21" spans="1:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="4"/>
       <c r="B21" s="5" t="s">
         <v>22</v>
@@ -1048,51 +1076,81 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A22" s="11"/>
-      <c r="B22" s="12"/>
-      <c r="C22" s="12"/>
-      <c r="D22" s="12"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="12"/>
-      <c r="H22" s="12"/>
-      <c r="I22" s="12"/>
-      <c r="J22" s="11"/>
-      <c r="K22" s="12"/>
-      <c r="L22" s="12"/>
-      <c r="M22" s="12"/>
-      <c r="N22" s="11"/>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B23" s="13"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="G23" s="13"/>
-      <c r="H23" s="13"/>
-      <c r="I23" s="13"/>
-      <c r="K23" s="13"/>
-      <c r="L23" s="13"/>
-      <c r="M23" s="13"/>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B24" s="25"/>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A22" s="21"/>
+      <c r="B22" s="22"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="21"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="22"/>
+      <c r="H22" s="22"/>
+      <c r="I22" s="22"/>
+      <c r="J22" s="21"/>
+      <c r="K22" s="22"/>
+      <c r="L22" s="22"/>
+      <c r="M22" s="22"/>
+      <c r="N22" s="21"/>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B23" s="23" t="s">
+        <v>27</v>
+      </c>
+      <c r="C23" s="23"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="23" t="s">
+        <v>28</v>
+      </c>
+      <c r="H23" s="23"/>
+      <c r="I23" s="23"/>
+      <c r="J23" s="24"/>
+      <c r="K23" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="L23" s="23"/>
+      <c r="M23" s="23"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B24" s="25" t="s">
+        <v>30</v>
+      </c>
       <c r="C24" s="25"/>
       <c r="D24" s="25"/>
-      <c r="G24" s="24"/>
-      <c r="H24" s="24"/>
-      <c r="I24" s="24"/>
-      <c r="K24" s="24"/>
-      <c r="L24" s="24"/>
-      <c r="M24" s="24"/>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B25" s="24"/>
-      <c r="C25" s="24"/>
-      <c r="D25" s="24"/>
+      <c r="E24" s="24"/>
+      <c r="F24" s="24"/>
+      <c r="G24" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="H24" s="26"/>
+      <c r="I24" s="26"/>
+      <c r="J24" s="24"/>
+      <c r="K24" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="L24" s="26"/>
+      <c r="M24" s="26"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B25" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="19">
+    <mergeCell ref="J1:N1"/>
+    <mergeCell ref="J2:N2"/>
+    <mergeCell ref="J3:N3"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="G23:I23"/>
+    <mergeCell ref="G24:I24"/>
+    <mergeCell ref="K23:M23"/>
+    <mergeCell ref="K24:M24"/>
+    <mergeCell ref="B24:D24"/>
     <mergeCell ref="A5:N5"/>
     <mergeCell ref="M6:N6"/>
     <mergeCell ref="A13:A14"/>
@@ -1102,9 +1160,6 @@
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="H13:J13"/>
     <mergeCell ref="K13:M13"/>
-    <mergeCell ref="J1:N1"/>
-    <mergeCell ref="J2:N2"/>
-    <mergeCell ref="J3:N3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="86" fitToHeight="0" orientation="landscape" r:id="rId1"/>

</xml_diff>